<commit_message>
Update HarborPoint_Winds of Fortune Template.xlsx
switched from winds SIP name to wind name
</commit_message>
<xml_diff>
--- a/data/HarborPoint_Winds of Fortune Template.xlsx
+++ b/data/HarborPoint_Winds of Fortune Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Probability Management\Portfolio Build\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E1BCB64-4ECD-4408-9209-1420DE51F024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{768BA7C6-4D39-4864-BE9A-1886C908F0CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{62E0E9A3-437D-464E-8FB6-CFA38D87EB32}"/>
   </bookViews>
@@ -77,25 +77,25 @@
     <t>PT</t>
   </si>
   <si>
-    <t>WIND1</t>
-  </si>
-  <si>
-    <t>WIND2</t>
-  </si>
-  <si>
-    <t>WIND3</t>
-  </si>
-  <si>
-    <t>WIND4</t>
-  </si>
-  <si>
-    <t>WIND5</t>
-  </si>
-  <si>
-    <t>WIND6</t>
-  </si>
-  <si>
-    <t>WIND7</t>
+    <t>Commercial Payer Mix Shift</t>
+  </si>
+  <si>
+    <t>Specialist Labor Availability</t>
+  </si>
+  <si>
+    <t>Medicare Rate Pressure</t>
+  </si>
+  <si>
+    <t>Local Employer Growth</t>
+  </si>
+  <si>
+    <t>Ambulatory Competition Intensity</t>
+  </si>
+  <si>
+    <t>Population Aging Rate</t>
+  </si>
+  <si>
+    <t>Behavioral Health Policy Expansion</t>
   </si>
 </sst>
 </file>

</xml_diff>